<commit_message>
Modification to test jenkins
</commit_message>
<xml_diff>
--- a/testdata/BookingData.xlsx
+++ b/testdata/BookingData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\eclipse-workspace\FlightBooking\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2EB1D5BB-9B69-4D32-AB98-3B343AD5AC8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{574FF644-2890-4E8D-ACBF-F568BA26A084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{664C9574-2777-4555-BCC8-F4C9E658CBD7}"/>
   </bookViews>
@@ -60,28 +60,28 @@
     <t>London</t>
   </si>
   <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>NY</t>
-  </si>
-  <si>
-    <t>CA</t>
-  </si>
-  <si>
-    <t>Street1</t>
-  </si>
-  <si>
-    <t>Street2</t>
-  </si>
-  <si>
-    <t>Mike</t>
-  </si>
-  <si>
     <t>Rome</t>
   </si>
   <si>
     <t>Paris</t>
+  </si>
+  <si>
+    <t>Prakhar</t>
+  </si>
+  <si>
+    <t>NCR</t>
+  </si>
+  <si>
+    <t>DELHI</t>
+  </si>
+  <si>
+    <t>Ravi</t>
+  </si>
+  <si>
+    <t>Noida</t>
+  </si>
+  <si>
+    <t>UP</t>
   </si>
 </sst>
 </file>
@@ -464,33 +464,33 @@
         <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F2">
-        <v>1111</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F3">
         <v>2222</v>

</xml_diff>